<commit_message>
Update September KPI with corrected Kurly delivery cost
Hot pack Market Kurly (Saetbyeol) shipping cost is 0 in the source
workbook, raising hot pack operating profit to 10,216,114 (36.1%) and
combined to 26,919,164 (19.6%).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U57HqgEQfdTuX1dvSuHD8X
</commit_message>
<xml_diff>
--- a/kpi/2026-09/2026-09_온라인_KPI.xlsx
+++ b/kpi/2026-09/2026-09_온라인_KPI.xlsx
@@ -643,7 +643,7 @@
         <v>28319705</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>9661714</v>
+        <v>10216114</v>
       </c>
       <c r="D6" s="6">
         <f>C6/B6</f>
@@ -667,7 +667,7 @@
         <v>0.08638730523499451</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>0.1647988211741613</v>
+        <v>0.1452223460661048</v>
       </c>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="6">
@@ -686,7 +686,7 @@
         <v>137007028</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>26364763</v>
+        <v>26919163</v>
       </c>
       <c r="D7" s="12">
         <f>C7/B7</f>
@@ -710,7 +710,7 @@
         <v>0.09663359751150868</v>
       </c>
       <c r="J7" s="12" t="n">
-        <v>0.1588225094555003</v>
+        <v>0.1547760017099269</v>
       </c>
       <c r="K7" s="11">
         <f>K5+K6</f>
@@ -2247,10 +2247,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>554400</v>
+        <v>0</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>1474520</v>
+        <v>2028920</v>
       </c>
       <c r="J3" s="6">
         <f>IFERROR(I3/C3,"-")</f>
@@ -3028,10 +3028,10 @@
         <v>1013127</v>
       </c>
       <c r="H19" s="11" t="n">
-        <v>4667054</v>
+        <v>4112654</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>9661714</v>
+        <v>10216114</v>
       </c>
       <c r="J19" s="12">
         <f>I19/C19</f>

</xml_diff>